<commit_message>
Separate policies and registers into individual files
- Split every multi-register workbook so each register is its own file
  (32 register files in registers/, including the Word AML Incident
  Register); remove the combined workbooks.
- Move the 12 policies into policies/.
- Remove the register field table from the Complaints Procedure so no
  policy contains register content; policies now reference each
  separate register file by name in their "Supporting registers"
  sections.
- Update register guidance text and SUMMARY.md accordingly.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185GJD35Lj4maZQfYQD6Tsw
</commit_message>
<xml_diff>
--- a/framework-templates/registers/Compliance_Breach_Log_v2.0_Template.xlsx
+++ b/framework-templates/registers/Compliance_Breach_Log_v2.0_Template.xlsx
@@ -768,10 +768,10 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="49" customHeight="1">
+    <row r="16" ht="34" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Personal data breaches are recorded in the Data Breach Log in the Data Protection Registers workbook, which covers ICO notification within 72 hours. Where a data breach is also a regulatory breach (for example a significant cyber incident), record it in both and cross-refer.</t>
+          <t>Personal data breaches are recorded in the separate Data Breach Log, which covers ICO notification within 72 hours. Where a data breach is also a regulatory breach (for example a significant cyber incident), record it in both and cross-refer.</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
     <row r="18" ht="49" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>Every breach must have remedial action with an owner and a deadline. Larger actions are tracked in the Corrective Action Log (in the Compliance Monitoring Tracker workbook) – record the reference here. Close a breach only when the root cause has been fixed and any affected customers have been put right.</t>
+          <t>Every breach must have remedial action with an owner and a deadline. Larger actions are tracked in the separate Corrective Action Log – record the reference here. Close a breach only when the root cause has been fixed and any affected customers have been put right.</t>
         </is>
       </c>
     </row>

</xml_diff>